<commit_message>
extra xf4 plots for appendix
</commit_message>
<xml_diff>
--- a/Extras/Wedge/wedge_data_2026-04-10.xlsx
+++ b/Extras/Wedge/wedge_data_2026-04-10.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\patri\projects\emma-openmc\Extras\Wedge\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/patrickpark/git-repos/emma-openmc/Extras/Wedge/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C97DF041-600A-46A8-9EE0-5D5D403F2AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C55BFEFE-3BEE-FB4F-8829-DE7569A35F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="30720" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="3" r:id="rId1"/>
@@ -7182,29 +7182,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C22416C2-1180-4450-A3B0-0B08DD9AEC85}">
   <dimension ref="A1:Q104"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
-    <col min="2" max="2" width="2.109375" customWidth="1"/>
-    <col min="3" max="5" width="12.21875" customWidth="1"/>
-    <col min="6" max="7" width="15.88671875" customWidth="1"/>
-    <col min="8" max="8" width="12.5546875" customWidth="1"/>
-    <col min="9" max="9" width="15.109375" customWidth="1"/>
-    <col min="10" max="10" width="2.77734375" customWidth="1"/>
+    <col min="2" max="2" width="2.1640625" customWidth="1"/>
+    <col min="3" max="5" width="12.1640625" customWidth="1"/>
+    <col min="6" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.5" customWidth="1"/>
+    <col min="9" max="9" width="15.1640625" customWidth="1"/>
+    <col min="10" max="10" width="2.83203125" customWidth="1"/>
     <col min="11" max="13" width="13.33203125" customWidth="1"/>
-    <col min="14" max="14" width="15.5546875" customWidth="1"/>
-    <col min="15" max="15" width="14.21875" customWidth="1"/>
-    <col min="16" max="16" width="12.21875" customWidth="1"/>
-    <col min="17" max="17" width="12.77734375" customWidth="1"/>
+    <col min="14" max="14" width="15.5" customWidth="1"/>
+    <col min="15" max="15" width="14.1640625" customWidth="1"/>
+    <col min="16" max="16" width="12.1640625" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C2" s="11" t="s">
         <v>2</v>
       </c>
@@ -7218,7 +7218,7 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C3" s="13" t="s">
         <v>4</v>
       </c>
@@ -7238,7 +7238,7 @@
       <c r="P3" s="16"/>
       <c r="Q3" s="16"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>0</v>
       </c>
@@ -7287,7 +7287,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>0.1</v>
       </c>
@@ -7334,7 +7334,7 @@
         <v>1.1566053404779838E-4</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>0.5</v>
       </c>
@@ -7381,7 +7381,7 @@
         <v>1.4663372036719969E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1</v>
       </c>
@@ -7428,7 +7428,7 @@
         <v>1.2067125581283931E-4</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>10</v>
       </c>
@@ -7475,7 +7475,7 @@
         <v>5.3733016877644728E-4</v>
       </c>
     </row>
-    <row r="9" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>25</v>
       </c>
@@ -7523,7 +7523,7 @@
         <v>1.3654161494401974E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>50</v>
       </c>
@@ -7570,7 +7570,7 @@
         <v>1.4086562192379159E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>75</v>
       </c>
@@ -7618,7 +7618,7 @@
         <v>1.5161165627240361E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>100</v>
       </c>
@@ -7665,7 +7665,7 @@
         <v>1.4295491548200695E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>150</v>
       </c>
@@ -7712,7 +7712,7 @@
         <v>1.3731787771009375E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>250</v>
       </c>
@@ -7760,7 +7760,7 @@
         <v>1.3837178252034666E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>500</v>
       </c>
@@ -7807,7 +7807,7 @@
         <v>1.9373993710566338E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>750</v>
       </c>
@@ -7855,7 +7855,7 @@
         <v>1.7381247050213394E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>999.99</v>
       </c>
@@ -7902,7 +7902,7 @@
         <v>1.4291594730581141E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C19" s="9" t="s">
         <v>5</v>
       </c>
@@ -7917,7 +7917,7 @@
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C20" s="13" t="s">
         <v>4</v>
       </c>
@@ -7937,7 +7937,7 @@
       <c r="P20" s="16"/>
       <c r="Q20" s="16"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>0</v>
       </c>
@@ -7986,7 +7986,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>0.1</v>
       </c>
@@ -8035,7 +8035,7 @@
         <v>6.3128152538764219E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>0.5</v>
       </c>
@@ -8082,7 +8082,7 @@
         <v>3.0980641245473535E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>1</v>
       </c>
@@ -8129,7 +8129,7 @@
         <v>2.9926223455543194E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>10</v>
       </c>
@@ -8176,7 +8176,7 @@
         <v>2.0807117833009201E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -8223,7 +8223,7 @@
         <v>4.8088408512878518E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>50</v>
       </c>
@@ -8270,7 +8270,7 @@
         <v>3.3931826596209033E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>75</v>
       </c>
@@ -8317,7 +8317,7 @@
         <v>4.3732957749830943E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>100</v>
       </c>
@@ -8364,7 +8364,7 @@
         <v>3.270987741553931E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>150</v>
       </c>
@@ -8411,7 +8411,7 @@
         <v>3.0120489033709811E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>250</v>
       </c>
@@ -8458,7 +8458,7 @@
         <v>2.4811355128425004E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>500</v>
       </c>
@@ -8505,7 +8505,7 @@
         <v>2.5334379936179344E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>750</v>
       </c>
@@ -8552,7 +8552,7 @@
         <v>2.2881645006526826E-3</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>999.99</v>
       </c>
@@ -8599,7 +8599,7 @@
         <v>2.0761752123647477E-3</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C36" s="9" t="s">
         <v>13</v>
       </c>
@@ -8614,7 +8614,7 @@
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C37" s="13" t="s">
         <v>4</v>
       </c>
@@ -8634,7 +8634,7 @@
       <c r="P37" s="16"/>
       <c r="Q37" s="16"/>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
         <v>0</v>
       </c>
@@ -8683,7 +8683,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>0.1</v>
       </c>
@@ -8732,7 +8732,7 @@
         <v>2.4692029617883636E-3</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>0.5</v>
       </c>
@@ -8779,7 +8779,7 @@
         <v>9.6145500722271619E-4</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>1</v>
       </c>
@@ -8826,7 +8826,7 @@
         <v>7.3061732078473008E-4</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>10</v>
       </c>
@@ -8873,7 +8873,7 @@
         <v>7.736996230761808E-4</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>25</v>
       </c>
@@ -8920,7 +8920,7 @@
         <v>2.657998552514734E-3</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>50</v>
       </c>
@@ -8967,7 +8967,7 @@
         <v>2.2733212468731513E-3</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>75</v>
       </c>
@@ -9014,7 +9014,7 @@
         <v>1.8192394881123154E-3</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>100</v>
       </c>
@@ -9061,7 +9061,7 @@
         <v>2.09604744411438E-3</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>150</v>
       </c>
@@ -9108,7 +9108,7 @@
         <v>1.9036453265773162E-3</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>250</v>
       </c>
@@ -9155,7 +9155,7 @@
         <v>2.08013448905876E-3</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>500</v>
       </c>
@@ -9202,7 +9202,7 @@
         <v>1.8774931839575925E-3</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>750</v>
       </c>
@@ -9249,7 +9249,7 @@
         <v>1.7528003368185298E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>999.99</v>
       </c>
@@ -9296,12 +9296,12 @@
         <v>1.5490415302505404E-3</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C54" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C55" s="11" t="s">
         <v>2</v>
       </c>
@@ -9315,7 +9315,7 @@
       <c r="M55" s="2"/>
       <c r="N55" s="2"/>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C56" s="13" t="s">
         <v>4</v>
       </c>
@@ -9335,7 +9335,7 @@
       <c r="P56" s="16"/>
       <c r="Q56" s="16"/>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A57" s="5" t="s">
         <v>0</v>
       </c>
@@ -9384,7 +9384,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>0.1</v>
       </c>
@@ -9431,7 +9431,7 @@
         <v>9.766545498253321E-5</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>0.5</v>
       </c>
@@ -9479,7 +9479,7 @@
         <v>1.3707596618126611E-4</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>1</v>
       </c>
@@ -9526,7 +9526,7 @@
         <v>1.385783590344851E-4</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>10</v>
       </c>
@@ -9574,7 +9574,7 @@
         <v>3.5291035880064285E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>25</v>
       </c>
@@ -9621,7 +9621,7 @@
         <v>1.5109184058008226E-3</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>50</v>
       </c>
@@ -9669,7 +9669,7 @@
         <v>1.3301552387791574E-3</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>75</v>
       </c>
@@ -9716,7 +9716,7 @@
         <v>1.353530062079468E-3</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>100</v>
       </c>
@@ -9764,7 +9764,7 @@
         <v>1.3216984553462278E-3</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>150</v>
       </c>
@@ -9805,7 +9805,7 @@
         <v>1.138865863749726E-3</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>250</v>
       </c>
@@ -9847,7 +9847,7 @@
         <v>1.1996852761766263E-3</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>500</v>
       </c>
@@ -9888,7 +9888,7 @@
         <v>1.7155928133229267E-3</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>750</v>
       </c>
@@ -9929,7 +9929,7 @@
         <v>1.2587483955646352E-3</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>999.99</v>
       </c>
@@ -9970,7 +9970,7 @@
         <v>1.4941713528427928E-3</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C72" s="9" t="s">
         <v>5</v>
       </c>
@@ -9985,7 +9985,7 @@
       <c r="M72" s="2"/>
       <c r="N72" s="2"/>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C73" s="13" t="s">
         <v>4</v>
       </c>
@@ -10005,7 +10005,7 @@
       <c r="P73" s="16"/>
       <c r="Q73" s="16"/>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
         <v>0</v>
       </c>
@@ -10054,7 +10054,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>0.1</v>
       </c>
@@ -10103,7 +10103,7 @@
         <v>1.4173467854162441E-3</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>0.5</v>
       </c>
@@ -10151,7 +10151,7 @@
         <v>6.1579904211881168E-4</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>1</v>
       </c>
@@ -10199,7 +10199,7 @@
         <v>4.5681987639143909E-4</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>10</v>
       </c>
@@ -10247,7 +10247,7 @@
         <v>7.1565365199815936E-4</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>25</v>
       </c>
@@ -10295,7 +10295,7 @@
         <v>2.2304176516532194E-3</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>50</v>
       </c>
@@ -10343,7 +10343,7 @@
         <v>2.0253690793008185E-3</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>75</v>
       </c>
@@ -10391,7 +10391,7 @@
         <v>1.664087211902877E-3</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>100</v>
       </c>
@@ -10439,7 +10439,7 @@
         <v>1.8410592624697934E-3</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>150</v>
       </c>
@@ -10481,7 +10481,7 @@
         <v>1.4505601412026115E-3</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>250</v>
       </c>
@@ -10523,7 +10523,7 @@
         <v>1.6119220123475947E-3</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>500</v>
       </c>
@@ -10565,7 +10565,7 @@
         <v>2.0148885303333877E-3</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>750</v>
       </c>
@@ -10606,7 +10606,7 @@
         <v>1.4722528853940004E-3</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>999.99</v>
       </c>
@@ -10647,7 +10647,7 @@
         <v>1.7820258962268976E-3</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C89" s="19" t="s">
         <v>13</v>
       </c>
@@ -10662,7 +10662,7 @@
       <c r="M89" s="2"/>
       <c r="N89" s="2"/>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C90" s="13" t="s">
         <v>4</v>
       </c>
@@ -10682,7 +10682,7 @@
       <c r="P90" s="16"/>
       <c r="Q90" s="16"/>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A91" s="5" t="s">
         <v>0</v>
       </c>
@@ -10731,7 +10731,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>0.1</v>
       </c>
@@ -10780,7 +10780,7 @@
         <v>1.6165722467163411E-3</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>0.5</v>
       </c>
@@ -10828,7 +10828,7 @@
         <v>7.2522325975314477E-4</v>
       </c>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>1</v>
       </c>
@@ -10876,7 +10876,7 @@
         <v>5.4736218274390727E-4</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>10</v>
       </c>
@@ -10924,7 +10924,7 @@
         <v>6.6793464964274413E-4</v>
       </c>
     </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>25</v>
       </c>
@@ -10972,7 +10972,7 @@
         <v>1.713396075801996E-3</v>
       </c>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>50</v>
       </c>
@@ -11020,7 +11020,7 @@
         <v>1.4512066100184763E-3</v>
       </c>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>75</v>
       </c>
@@ -11068,7 +11068,7 @@
         <v>1.3709912639735175E-3</v>
       </c>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>100</v>
       </c>
@@ -11116,7 +11116,7 @@
         <v>1.353566839850045E-3</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>150</v>
       </c>
@@ -11158,7 +11158,7 @@
         <v>1.2434009620595613E-3</v>
       </c>
     </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>250</v>
       </c>
@@ -11200,7 +11200,7 @@
         <v>1.3435343559292461E-3</v>
       </c>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>500</v>
       </c>
@@ -11242,7 +11242,7 @@
         <v>1.2367835060891773E-3</v>
       </c>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>750</v>
       </c>
@@ -11283,7 +11283,7 @@
         <v>1.151186180212625E-3</v>
       </c>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>999.99</v>
       </c>

</xml_diff>